<commit_message>
Atualiza convite: família, macarronada, cores alegres, data, local e acompanhantes
Agent-Logs-Url: https://github.com/eronbfr/Convite_Especial/sessions/307c8c6d-6dfe-42d5-a15e-c420bab4bc47

Co-authored-by: eronbfr <270444003+eronbfr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lista_de_presenca.xlsx
+++ b/lista_de_presenca.xlsx
@@ -11,12 +11,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Nome Completo</t>
   </si>
   <si>
     <t>Acompanhantes</t>
+  </si>
+  <si>
+    <t>Nomes dos Acompanhantes</t>
   </si>
   <si>
     <t>Mensagem</t>
@@ -403,16 +406,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="3" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -425,6 +428,9 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>